<commit_message>
Add note for Month 7 partial data in summary sheet
</commit_message>
<xml_diff>
--- a/NovaMart_Sales_Raw-Project.xlsx
+++ b/NovaMart_Sales_Raw-Project.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\data-analyst-projects\novamart-sales-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B53B1A8-D458-48F8-BD5C-16CA21F0FBB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D607786-32F0-491B-BD18-B765D6150C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pivot1" sheetId="5" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="138">
   <si>
     <t>Order ID</t>
   </si>
@@ -466,6 +466,9 @@
   </si>
   <si>
     <t>On Target</t>
+  </si>
+  <si>
+    <t>Month 7 - Partial month — growth figure not representative</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1210,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[NovaMart_Sales_Raw-Claude-Practice-plan.xlsx]Pivot2!PivotTable2</c:name>
+    <c:name>[NovaMart_Sales_Raw-Project.xlsx]Pivot2!PivotTable2</c:name>
     <c:fmtId val="0"/>
   </c:pivotSource>
   <c:chart>
@@ -1615,7 +1618,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[NovaMart_Sales_Raw-Claude-Practice-plan.xlsx]Pivot2!PivotTable2</c:name>
+    <c:name>[NovaMart_Sales_Raw-Project.xlsx]Pivot2!PivotTable2</c:name>
     <c:fmtId val="4"/>
   </c:pivotSource>
   <c:chart>
@@ -8219,6 +8222,9 @@
         <f t="shared" si="1"/>
         <v>-1</v>
       </c>
+      <c r="L8" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="L10" s="12"/>

</xml_diff>